<commit_message>
[PROGRAMMER] Plan68 gamma-B: enemy move speed relative multiplier (player=1.0, base 210) + SHEEP align
</commit_message>
<xml_diff>
--- a/Design/Data/ReEchoEncounterData.xlsx
+++ b/Design/Data/ReEchoEncounterData.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stages" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Encounters" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EncounterWaves" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SpawnProfiles" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SpawnPolicy" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_ExportMap" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Stages" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Encounters" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="EncounterWaves" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="SpawnProfiles" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="SpawnPolicy" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="_ExportMap" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
 </workbook>
@@ -172,9 +172,7 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment/>
-    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -639,6 +637,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="15" customHeight="1">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -954,6 +953,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="15" customHeight="1">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -1700,6 +1700,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="15" customHeight="1">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -2756,7 +2757,7 @@
       </c>
       <c r="H25" s="26" t="inlineStr">
         <is>
-          <t>M_TimeGuard</t>
+          <t>M_SHEEP</t>
         </is>
       </c>
       <c r="I25" s="26" t="inlineStr">
@@ -2829,6 +2830,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="15" customHeight="1">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -3184,6 +3186,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="15" customHeight="1">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -3354,27 +3357,27 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="inlineStr">
+      <c r="A1" s="5" t="inlineStr">
         <is>
           <t>SheetName</t>
         </is>
       </c>
-      <c r="B1" s="4" t="inlineStr">
+      <c r="B1" s="5" t="inlineStr">
         <is>
           <t>TableName</t>
         </is>
       </c>
-      <c r="C1" s="4" t="inlineStr">
+      <c r="C1" s="5" t="inlineStr">
         <is>
           <t>AdapterVersion</t>
         </is>
       </c>
-      <c r="D1" s="4" t="inlineStr">
+      <c r="D1" s="5" t="inlineStr">
         <is>
           <t>OutputCsv</t>
         </is>
       </c>
-      <c r="E1" s="4" t="inlineStr">
+      <c r="E1" s="5" t="inlineStr">
         <is>
           <t>SortKey</t>
         </is>

</xml_diff>

<commit_message>
[PROGRAMMER] Implement stage scene switching and camera edge limits
</commit_message>
<xml_diff>
--- a/Design/Data/ReEchoEncounterData.xlsx
+++ b/Design/Data/ReEchoEncounterData.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet name="Stages" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Encounters" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="EncounterWaves" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="SpawnProfiles" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="SpawnPolicy" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="_ExportMap" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stages" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Encounters" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EncounterWaves" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SpawnProfiles" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SpawnPolicy" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_ExportMap" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
 </workbook>
@@ -637,7 +637,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="15" customHeight="1">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -706,7 +705,7 @@
       </c>
       <c r="C4" s="20" t="inlineStr">
         <is>
-          <t>Level00</t>
+          <t>SC01</t>
         </is>
       </c>
       <c r="D4" s="20" t="n">
@@ -755,7 +754,7 @@
       </c>
       <c r="C5" s="23" t="inlineStr">
         <is>
-          <t>Level00</t>
+          <t>SC02</t>
         </is>
       </c>
       <c r="D5" s="23" t="n">
@@ -804,7 +803,7 @@
       </c>
       <c r="C6" s="23" t="inlineStr">
         <is>
-          <t>Level00</t>
+          <t>SC03</t>
         </is>
       </c>
       <c r="D6" s="23" t="n">
@@ -853,7 +852,7 @@
       </c>
       <c r="C7" s="26" t="inlineStr">
         <is>
-          <t>Level00</t>
+          <t>SC04</t>
         </is>
       </c>
       <c r="D7" s="26" t="n">
@@ -953,7 +952,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="15" customHeight="1">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -1700,7 +1698,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="15" customHeight="1">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -2830,7 +2827,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="15" customHeight="1">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -3186,7 +3182,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="15" customHeight="1">
       <c r="A3" s="5" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
[PROGRAMMER] 修复 Boss 固定出生位置
</commit_message>
<xml_diff>
--- a/Design/Data/ReEchoEncounterData.xlsx
+++ b/Design/Data/ReEchoEncounterData.xlsx
@@ -363,7 +363,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="tblSpawnProfiles" displayName="tblSpawnProfiles" ref="A3:M7" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="tblSpawnProfiles" displayName="tblSpawnProfiles" ref="A3:M8" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <tableColumns count="13">
     <tableColumn id="1" name="Id"/>
     <tableColumn id="2" name="EnemyRole"/>
@@ -2889,12 +2889,12 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M7"/>
+  <dimension ref="A1:M8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40.5" customWidth="1" min="1" max="1"/>
@@ -3214,31 +3214,88 @@
         </is>
       </c>
     </row>
+    <row r="8" ht="15" customHeight="1">
+      <c r="A8" s="25" t="inlineStr">
+        <is>
+          <t>Spawn.Boss</t>
+        </is>
+      </c>
+      <c r="B8" s="26" t="inlineStr">
+        <is>
+          <t>Boss</t>
+        </is>
+      </c>
+      <c r="C8" s="26" t="inlineStr">
+        <is>
+          <t>M_SHEEP</t>
+        </is>
+      </c>
+      <c r="D8" s="26">
+        <v>700</v>
+      </c>
+      <c r="E8" s="26">
+        <v>950</v>
+      </c>
+      <c r="F8" s="26">
+        <v>220</v>
+      </c>
+      <c r="G8" s="26">
+        <v>0.9</v>
+      </c>
+      <c r="H8" s="26" t="inlineStr">
+        <is>
+          <t>NormalAroundAnchor</t>
+        </is>
+      </c>
+      <c r="I8" s="26" t="inlineStr">
+        <is>
+          <t>Explicit</t>
+        </is>
+      </c>
+      <c r="J8" s="26" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="K8" s="26" t="inlineStr">
+        <is>
+          <t>刷怪规则</t>
+        </is>
+      </c>
+      <c r="L8" s="26">
+        <v>13</v>
+      </c>
+      <c r="M8" s="27" t="inlineStr">
+        <is>
+          <t>Boss使用双锚动态出生；不再使用固定坐标</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="0" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="0" formatCells="1" formatRows="1" sort="1"/>
   <mergeCells count="1">
     <mergeCell ref="A1:M1"/>
   </mergeCells>
   <dataValidations count="5">
-    <dataValidation sqref="B4:B7" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
-      <formula1>"Melee,Ranged,Elite,BossReinforcement"</formula1>
+    <dataValidation sqref="B4:B8" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
+      <formula1>"Melee,Ranged,Elite,BossReinforcement,Boss"</formula1>
     </dataValidation>
-    <dataValidation sqref="C4:C7" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
-      <formula1>"M_SLIME,M_RABBIT,M_FOX,M_TimeGuard"</formula1>
+    <dataValidation sqref="C4:C8" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
+      <formula1>"M_SLIME,M_RABBIT,M_FOX,M_TimeGuard,M_SHEEP"</formula1>
     </dataValidation>
-    <dataValidation sqref="H4:H7" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
+    <dataValidation sqref="H4:H8" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
       <formula1>"NormalAroundAnchor"</formula1>
     </dataValidation>
-    <dataValidation sqref="I4:I7" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
+    <dataValidation sqref="I4:I8" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
       <formula1>"Explicit,UseEnemyRole"</formula1>
     </dataValidation>
-    <dataValidation sqref="J4:J7" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
+    <dataValidation sqref="J4:J8" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
       <formula1>"true,false"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+    <tablePart r:id="rId1"/>
   </tableParts>
 </worksheet>
 </file>

</xml_diff>